<commit_message>
Update tampilan halaman about
</commit_message>
<xml_diff>
--- a/data/kbli_populer_riau2.xlsx
+++ b/data/kbli_populer_riau2.xlsx
@@ -9225,7 +9225,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>1676</v>
       </c>
@@ -15560,7 +15560,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="224" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A224" s="6" t="s">
         <v>1844</v>
       </c>
@@ -30288,7 +30288,7 @@
         <v>1919</v>
       </c>
     </row>
-    <row r="646" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="646" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A646" s="6" t="s">
         <v>1845</v>
       </c>
@@ -30323,7 +30323,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="647" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="647" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A647" s="6" t="s">
         <v>1845</v>
       </c>
@@ -30883,7 +30883,7 @@
         <v>2002</v>
       </c>
     </row>
-    <row r="663" spans="1:11" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="663" spans="1:11" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A663" s="6" t="s">
         <v>5</v>
       </c>
@@ -31548,7 +31548,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="682" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="682" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A682" s="6" t="s">
         <v>2022</v>
       </c>
@@ -31583,7 +31583,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="683" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="683" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A683" s="6" t="s">
         <v>2022</v>
       </c>
@@ -32983,7 +32983,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="723" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="723" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A723" s="6" t="s">
         <v>2022</v>
       </c>
@@ -35573,7 +35573,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="797" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="797" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A797" s="6" t="s">
         <v>2023</v>
       </c>
@@ -35713,7 +35713,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="801" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="801" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A801" s="6" t="s">
         <v>2023</v>
       </c>
@@ -35853,7 +35853,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="805" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="805" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A805" s="6" t="s">
         <v>2023</v>
       </c>
@@ -36728,7 +36728,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="830" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="830" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A830" s="6" t="s">
         <v>2023</v>
       </c>
@@ -38513,7 +38513,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="881" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="881" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A881" s="6" t="s">
         <v>2023</v>
       </c>
@@ -38548,7 +38548,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="882" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="882" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A882" s="6" t="s">
         <v>2023</v>
       </c>
@@ -41103,7 +41103,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="955" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="955" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A955" s="6" t="s">
         <v>2024</v>
       </c>
@@ -41313,7 +41313,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="961" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="961" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A961" s="6" t="s">
         <v>2024</v>
       </c>
@@ -41348,7 +41348,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="962" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="962" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A962" s="6" t="s">
         <v>2024</v>
       </c>
@@ -43961,7 +43961,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="1037" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="1037" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A1037" s="6" t="s">
         <v>16</v>
       </c>
@@ -44057,7 +44057,7 @@
         <v>2060</v>
       </c>
     </row>
-    <row r="1040" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="1040" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A1040" s="6" t="s">
         <v>16</v>
       </c>
@@ -44220,7 +44220,7 @@
         <v>2075</v>
       </c>
     </row>
-    <row r="1045" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="1045" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A1045" s="6" t="s">
         <v>16</v>
       </c>
@@ -44459,7 +44459,7 @@
         <v>2098</v>
       </c>
     </row>
-    <row r="1052" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+    <row r="1052" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A1052" s="6" t="s">
         <v>16</v>
       </c>
@@ -44599,7 +44599,7 @@
         <v>2111</v>
       </c>
     </row>
-    <row r="1056" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="1056" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A1056" s="6" t="s">
         <v>16</v>
       </c>
@@ -44914,7 +44914,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="1065" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="1065" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A1065" s="6" t="s">
         <v>24</v>
       </c>
@@ -46804,7 +46804,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="1119" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="1119" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1119" s="6" t="s">
         <v>2266</v>
       </c>
@@ -47259,7 +47259,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="1132" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="1132" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1132" s="6" t="s">
         <v>2266</v>
       </c>
@@ -49359,7 +49359,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="1192" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="1192" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A1192" s="6" t="s">
         <v>2266</v>
       </c>
@@ -53244,7 +53244,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="1303" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="1303" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A1303" s="6" t="s">
         <v>2278</v>
       </c>
@@ -53279,7 +53279,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="1304" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="1304" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A1304" s="6" t="s">
         <v>2278</v>
       </c>
@@ -55764,7 +55764,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="1375" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="1375" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A1375" s="6" t="s">
         <v>41</v>
       </c>
@@ -55869,7 +55869,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="1378" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="1378" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1378" s="6" t="s">
         <v>41</v>
       </c>
@@ -58214,7 +58214,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="1445" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="1445" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1445" s="6" t="s">
         <v>81</v>
       </c>
@@ -61294,7 +61294,7 @@
         <v>2288</v>
       </c>
     </row>
-    <row r="1533" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+    <row r="1533" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A1533" s="6" t="s">
         <v>2283</v>
       </c>
@@ -61679,7 +61679,7 @@
         <v>2327</v>
       </c>
     </row>
-    <row r="1544" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="1544" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1544" s="6" t="s">
         <v>2283</v>
       </c>
@@ -61819,7 +61819,7 @@
         <v>2342</v>
       </c>
     </row>
-    <row r="1548" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="1548" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A1548" s="6" t="s">
         <v>2283</v>
       </c>
@@ -62064,7 +62064,7 @@
         <v>2368</v>
       </c>
     </row>
-    <row r="1555" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="1555" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1555" s="6" t="s">
         <v>2283</v>
       </c>
@@ -62169,7 +62169,7 @@
         <v>2381</v>
       </c>
     </row>
-    <row r="1558" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="1558" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1558" s="6" t="s">
         <v>2376</v>
       </c>

</xml_diff>